<commit_message>
feat: update pipeline status to reflect running state and current agent activity
</commit_message>
<xml_diff>
--- a/outputs/schedule_kwality.xlsx
+++ b/outputs/schedule_kwality.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,11 +64,15 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <color rgb="00374151"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +121,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F0F0F5"/>
       </patternFill>
     </fill>
@@ -147,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -178,6 +187,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -545,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -631,8 +643,22 @@
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Mrigakshi Jaiswal
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
@@ -641,7 +667,14 @@
           <t>07:30</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Atulan Purohit
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -667,7 +700,14 @@
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
@@ -679,12 +719,19 @@
       <c r="B5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Anisha Shah
+Bret Saldanha
 32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
@@ -693,16 +740,7 @@
 []</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Raunak Khemuka
-33% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -710,6 +748,8 @@
 []</t>
         </is>
       </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
@@ -718,33 +758,40 @@
           <t>08:15</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Amped Up!
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
 Cauveri Vikrant
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle Express
+Mrigakshi Jaiswal
+43% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -773,13 +820,20 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>FIT
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n"/>
+          <t>Barre 57
+Karanvir Bhatia
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Rohan Dahima
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
@@ -789,14 +843,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Anisha Shah
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
@@ -816,14 +863,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Richard D'Costa
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -833,13 +873,20 @@
 []</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Cauveri Vikrant
+31% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Rohan Dahima
-63% pred | 0% hist
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+55% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -852,20 +899,27 @@
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Karanvir Bhatia
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Barre 57
+Vivaran Dhasmana
+50% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Rohan Dahima
-56% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Vivaran Dhasmana
-69% pred | 0% hist
+38% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -880,14 +934,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-29% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="7" t="inlineStr">
@@ -907,25 +954,32 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Reshma Sharma
+Anisha Shah
 44% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Reshma Sharma
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Karanvir Bhatia
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
     </row>
@@ -935,15 +989,15 @@
           <t>10:15</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
-Anisha Shah
-41% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -956,9 +1010,9 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>PowerCycle Express
-Reshma Sharma
-63% pred | 0% hist
+          <t>PowerCycle
+Rohan Dahima
+90% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -987,7 +1041,14 @@
 []</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Cauveri Vikrant
+48% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
@@ -998,7 +1059,14 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Reshma Sharma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Mat 57
@@ -1008,7 +1076,14 @@
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Atulan Purohit
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Full Body)
@@ -1039,14 +1114,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1055,7 +1123,14 @@
         </is>
       </c>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -1069,48 +1144,43 @@
       <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
-Atulan Purohit
+Reshma Sharma
 79% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+60% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Cauveri Vikrant
-100% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -1118,16 +1188,7 @@
 []</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
       <c r="H19" s="6" t="n"/>
@@ -1135,30 +1196,37 @@
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Recovery
+Karanvir Bhatia
+25% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
 Bret Saldanha
@@ -1167,100 +1235,100 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>17:45</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Vivaran Dhasmana
-40% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-44% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-    </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Vivaran Dhasmana
-31% pred | 0% hist
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57 Express
+Pranjali Jain
+67% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+44% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="n"/>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Bret Saldanha
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Anisha Shah
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Pull)
+Reshma Sharma
+63% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Mrigakshi Jaiswal
+86% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Bret Saldanha
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Karan Bhatia
-34% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="52" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Pranjali Jain
+32% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre Plus
-Karanvir Bhatia
-26% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="6" t="n"/>
@@ -1268,42 +1336,56 @@
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-47% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre Plus
+Raunak Khemuka
+26% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
     </row>
     <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Karanvir Bhatia
-85% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Anmol Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Mat 57
 Pranjali Jain
@@ -1311,33 +1393,40 @@
 []</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab
-Pranjali Jain
-43% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Trainer's Choice
+Anisha Shah
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>FIT
-Vivaran Dhasmana
+Reshma Sharma
 52% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Reshma Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
 Mrigakshi Jaiswal
@@ -1345,58 +1434,9 @@
 []</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-51% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Raunak Khemuka
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1412,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1498,8 +1538,22 @@
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Mrigakshi Jaiswal
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
@@ -1508,7 +1562,14 @@
           <t>07:30</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Atulan Purohit
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -1534,7 +1595,14 @@
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
@@ -1546,12 +1614,19 @@
       <c r="B5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Anisha Shah
+Bret Saldanha
 32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
@@ -1560,16 +1635,7 @@
 []</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Raunak Khemuka
-33% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -1577,6 +1643,8 @@
 []</t>
         </is>
       </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
@@ -1585,33 +1653,40 @@
           <t>08:15</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Amped Up!
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
 Cauveri Vikrant
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle Express
+Mrigakshi Jaiswal
+43% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -1640,13 +1715,20 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>FIT
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n"/>
+          <t>Barre 57
+Karanvir Bhatia
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Rohan Dahima
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
@@ -1656,14 +1738,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Anisha Shah
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
@@ -1683,14 +1758,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Richard D'Costa
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -1700,13 +1768,20 @@
 []</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Cauveri Vikrant
+31% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Rohan Dahima
-63% pred | 0% hist
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+55% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1719,20 +1794,27 @@
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Karanvir Bhatia
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Barre 57
+Vivaran Dhasmana
+50% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Rohan Dahima
-56% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Vivaran Dhasmana
-69% pred | 0% hist
+38% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1747,14 +1829,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-29% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="7" t="inlineStr">
@@ -1774,25 +1849,32 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Reshma Sharma
+Anisha Shah
 44% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Reshma Sharma
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Karanvir Bhatia
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
     </row>
@@ -1802,15 +1884,15 @@
           <t>10:15</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
-Anisha Shah
-41% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -1823,9 +1905,9 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>PowerCycle Express
-Reshma Sharma
-63% pred | 0% hist
+          <t>PowerCycle
+Rohan Dahima
+90% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1854,7 +1936,14 @@
 []</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Cauveri Vikrant
+48% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
@@ -1865,7 +1954,14 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Reshma Sharma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Mat 57
@@ -1875,7 +1971,14 @@
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Atulan Purohit
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Full Body)
@@ -1906,14 +2009,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1922,7 +2018,14 @@
         </is>
       </c>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -1936,48 +2039,43 @@
       <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
-Atulan Purohit
+Reshma Sharma
 79% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+60% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Cauveri Vikrant
-100% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -1985,16 +2083,7 @@
 []</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
       <c r="H19" s="6" t="n"/>
@@ -2002,30 +2091,37 @@
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Recovery
+Karanvir Bhatia
+25% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
 Bret Saldanha
@@ -2034,100 +2130,100 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>17:45</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Vivaran Dhasmana
-40% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-44% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-    </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Vivaran Dhasmana
-31% pred | 0% hist
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57 Express
+Pranjali Jain
+67% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+44% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="n"/>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Bret Saldanha
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Anisha Shah
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Pull)
+Reshma Sharma
+63% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Mrigakshi Jaiswal
+86% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Bret Saldanha
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Karan Bhatia
-34% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="52" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Pranjali Jain
+32% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre Plus
-Karanvir Bhatia
-26% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="6" t="n"/>
@@ -2135,42 +2231,56 @@
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-47% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre Plus
+Raunak Khemuka
+26% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
     </row>
     <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Karanvir Bhatia
-85% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Anmol Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Mat 57
 Pranjali Jain
@@ -2178,33 +2288,40 @@
 []</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab
-Pranjali Jain
-43% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Trainer's Choice
+Anisha Shah
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>FIT
-Vivaran Dhasmana
+Reshma Sharma
 52% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Reshma Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
 Mrigakshi Jaiswal
@@ -2212,58 +2329,9 @@
 []</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-51% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Raunak Khemuka
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2279,7 +2347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2365,8 +2433,22 @@
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Mrigakshi Jaiswal
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
@@ -2375,7 +2457,14 @@
           <t>07:30</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Atulan Purohit
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -2401,7 +2490,14 @@
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
@@ -2413,12 +2509,19 @@
       <c r="B5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Anisha Shah
+Bret Saldanha
 32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
@@ -2427,16 +2530,7 @@
 []</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Raunak Khemuka
-33% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -2444,6 +2538,8 @@
 []</t>
         </is>
       </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
@@ -2452,33 +2548,40 @@
           <t>08:15</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Amped Up!
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
 Cauveri Vikrant
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+45% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle Express
+Mrigakshi Jaiswal
+43% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -2507,13 +2610,20 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>FIT
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n"/>
+          <t>Barre 57
+Karanvir Bhatia
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Rohan Dahima
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
@@ -2523,14 +2633,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Anisha Shah
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
@@ -2550,14 +2653,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Richard D'Costa
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -2567,13 +2663,20 @@
 []</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Cauveri Vikrant
+31% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Rohan Dahima
-63% pred | 0% hist
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+55% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -2586,20 +2689,27 @@
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Karanvir Bhatia
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Barre 57
+Vivaran Dhasmana
+50% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
 Rohan Dahima
-56% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab (Push)
-Vivaran Dhasmana
-69% pred | 0% hist
+38% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -2614,14 +2724,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-29% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="7" t="inlineStr">
@@ -2641,25 +2744,32 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Reshma Sharma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>PowerCycle Express
-Reshma Sharma
+Anisha Shah
 44% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Reshma Sharma
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Karanvir Bhatia
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
     </row>
@@ -2669,15 +2779,15 @@
           <t>10:15</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
-Anisha Shah
-41% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Vivaran Dhasmana
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -2690,9 +2800,9 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>PowerCycle Express
-Reshma Sharma
-63% pred | 0% hist
+          <t>PowerCycle
+Rohan Dahima
+90% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -2721,7 +2831,14 @@
 []</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Cauveri Vikrant
+48% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
@@ -2732,7 +2849,14 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Reshma Sharma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Mat 57
@@ -2742,7 +2866,14 @@
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Atulan Purohit
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Full Body)
@@ -2773,14 +2904,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -2789,7 +2913,14 @@
         </is>
       </c>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
           <t>FIT
@@ -2803,48 +2934,43 @@
       <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
-Atulan Purohit
+Reshma Sharma
 79% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-52% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Vivaran Dhasmana
+60% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Cauveri Vikrant
-100% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Barre 57
 Rohan Dahima
@@ -2852,16 +2978,7 @@
 []</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
       <c r="H19" s="6" t="n"/>
@@ -2869,30 +2986,37 @@
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Mat 57
-Mrigakshi Jaiswal
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Recovery
+Karanvir Bhatia
+25% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>PowerCycle
 Bret Saldanha
@@ -2901,100 +3025,100 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>17:45</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Vivaran Dhasmana
-40% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Pranjali Jain
-44% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-    </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Vivaran Dhasmana
-31% pred | 0% hist
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57 Express
+Pranjali Jain
+67% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Pranjali Jain
+44% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="n"/>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Bret Saldanha
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Full Body)
+Anisha Shah
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Strength Lab (Pull)
+Reshma Sharma
+63% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Mrigakshi Jaiswal
+86% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Cauveri Vikrant
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Barre 57
+Bret Saldanha
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Karan Bhatia
-34% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="52" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>FIT
+Pranjali Jain
+32% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre Plus
-Karanvir Bhatia
-26% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="6" t="n"/>
@@ -3002,42 +3126,56 @@
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57
-Rohan Dahima
-47% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Cardio Barre Plus
+Raunak Khemuka
+26% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
     </row>
     <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle
-Karanvir Bhatia
-85% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>PowerCycle
+Anmol Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Mat 57
 Pranjali Jain
@@ -3045,33 +3183,40 @@
 []</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Strength Lab
-Pranjali Jain
-43% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Trainer's Choice
+Anisha Shah
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>FIT
-Vivaran Dhasmana
+Reshma Sharma
 52% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
+Reshma Sharma
+42% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Strength Lab (Pull)
 Mrigakshi Jaiswal
@@ -3079,58 +3224,9 @@
 []</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>PowerCycle Express
-Karan Bhatia
-51% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Trainer's Choice
-Raunak Khemuka
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pranjali Jain
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>